<commit_message>
Changes to be committed: 	deleted:    "descriptions/~$\320\232\320\275\320\270\320\263\320\2601.xlsx" 	modified:   "descriptions/\320\232\320\275\320\270\320\263\320\2601.xlsx" 	modified:   temp/datahandler/cocapi.py 	renamed:    temp/config.py -> temp/datahandler/config.py 	new file:   temp/documentation/description.txt 	modified:   temp/documentation/jsonstorage/instructions.txt
</commit_message>
<xml_diff>
--- a/descriptions/Книга1.xlsx
+++ b/descriptions/Книга1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terry\Documents\CODING\DB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\terry\Documents\CODING\DB\descriptions\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
   <si>
     <t>#2V2LRCL</t>
   </si>
@@ -81,13 +81,66 @@
   </si>
   <si>
     <t>Upgrades started</t>
+  </si>
+  <si>
+    <t>Тег</t>
+  </si>
+  <si>
+    <t>дата</t>
+  </si>
+  <si>
+    <t>ИК</t>
+  </si>
+  <si>
+    <t>войска</t>
+  </si>
+  <si>
+    <t>дал</t>
+  </si>
+  <si>
+    <t>получил</t>
+  </si>
+  <si>
+    <t>улучшения</t>
+  </si>
+  <si>
+    <t>золото столицы</t>
+  </si>
+  <si>
+    <t>кв</t>
+  </si>
+  <si>
+    <t>рейды</t>
+  </si>
+  <si>
+    <t>атаки</t>
+  </si>
+  <si>
+    <t>лвк</t>
+  </si>
+  <si>
+    <t>№</t>
+  </si>
+  <si>
+    <t>Итог</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00\ _₽_-;\-* #,##0.00\ _₽_-;_-* &quot;-&quot;??\ _₽_-;_-@_-"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,7 +158,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -199,11 +252,69 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -250,11 +361,71 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Финансовый" xfId="1" builtinId="3"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -530,13 +701,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B17:O20"/>
+  <dimension ref="A17:O65"/>
   <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="12.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B17" s="13" t="s">
         <v>3</v>
       </c>
@@ -554,7 +725,7 @@
       <c r="N17" s="14"/>
       <c r="O17" s="15"/>
     </row>
-    <row r="18" spans="2:15" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="10" t="s">
         <v>4</v>
       </c>
@@ -598,7 +769,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B19" s="3" t="s">
         <v>0</v>
       </c>
@@ -644,7 +815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B20" s="7" t="s">
         <v>17</v>
       </c>
@@ -662,10 +833,1141 @@
       <c r="N20" s="8"/>
       <c r="O20" s="9"/>
     </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" s="4"/>
+      <c r="B32" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
+      <c r="I32" s="14"/>
+      <c r="J32" s="14"/>
+      <c r="K32" s="15"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B33" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="E33" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="G33" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="H33" s="16"/>
+      <c r="I33" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J33" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K33" s="18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B34" s="27"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H34" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I34" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="J34" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="K34" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B35" s="28">
+        <v>1</v>
+      </c>
+      <c r="C35" s="24">
+        <v>46087</v>
+      </c>
+      <c r="D35" s="21">
+        <v>0</v>
+      </c>
+      <c r="E35" s="22">
+        <v>0</v>
+      </c>
+      <c r="F35" s="21">
+        <v>500</v>
+      </c>
+      <c r="G35" s="21">
+        <f ca="1">RANDBETWEEN(0,100)</f>
+        <v>63</v>
+      </c>
+      <c r="H35" s="21">
+        <f ca="1">RANDBETWEEN(0,100)</f>
+        <v>20</v>
+      </c>
+      <c r="I35" s="21">
+        <v>6</v>
+      </c>
+      <c r="J35" s="21">
+        <v>0</v>
+      </c>
+      <c r="K35" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="4"/>
+      <c r="B36" s="29">
+        <v>2</v>
+      </c>
+      <c r="C36" s="31">
+        <v>46086</v>
+      </c>
+      <c r="D36" s="4">
+        <v>0</v>
+      </c>
+      <c r="E36" s="18">
+        <v>1</v>
+      </c>
+      <c r="F36" s="4">
+        <v>500</v>
+      </c>
+      <c r="G36" s="4">
+        <f ca="1">RANDBETWEEN(0,100)</f>
+        <v>54</v>
+      </c>
+      <c r="H36" s="4">
+        <f ca="1">RANDBETWEEN(0,100)</f>
+        <v>98</v>
+      </c>
+      <c r="I36" s="4">
+        <v>0</v>
+      </c>
+      <c r="J36" s="4">
+        <v>0</v>
+      </c>
+      <c r="K36" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="4"/>
+      <c r="B37" s="29">
+        <v>3</v>
+      </c>
+      <c r="C37" s="31">
+        <v>46085</v>
+      </c>
+      <c r="D37" s="4">
+        <v>0</v>
+      </c>
+      <c r="E37" s="18">
+        <v>0</v>
+      </c>
+      <c r="F37" s="4">
+        <v>500</v>
+      </c>
+      <c r="G37" s="4">
+        <f t="shared" ref="G37:H63" ca="1" si="0">RANDBETWEEN(0,100)</f>
+        <v>31</v>
+      </c>
+      <c r="H37" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="I37" s="4">
+        <v>0</v>
+      </c>
+      <c r="J37" s="4">
+        <v>0</v>
+      </c>
+      <c r="K37" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="4"/>
+      <c r="B38" s="29">
+        <v>4</v>
+      </c>
+      <c r="C38" s="31">
+        <v>46084</v>
+      </c>
+      <c r="D38" s="4">
+        <v>0</v>
+      </c>
+      <c r="E38" s="18">
+        <v>0</v>
+      </c>
+      <c r="F38" s="4">
+        <v>500</v>
+      </c>
+      <c r="G38" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>77</v>
+      </c>
+      <c r="H38" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>57</v>
+      </c>
+      <c r="I38" s="4">
+        <v>0</v>
+      </c>
+      <c r="J38" s="4">
+        <v>0</v>
+      </c>
+      <c r="K38" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" s="4"/>
+      <c r="B39" s="29">
+        <v>5</v>
+      </c>
+      <c r="C39" s="31">
+        <v>46083</v>
+      </c>
+      <c r="D39" s="4">
+        <v>0</v>
+      </c>
+      <c r="E39" s="18">
+        <v>1</v>
+      </c>
+      <c r="F39" s="4">
+        <v>500</v>
+      </c>
+      <c r="G39" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="H39" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>39</v>
+      </c>
+      <c r="I39" s="4">
+        <v>0</v>
+      </c>
+      <c r="J39" s="4">
+        <v>2</v>
+      </c>
+      <c r="K39" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="4"/>
+      <c r="B40" s="29">
+        <v>6</v>
+      </c>
+      <c r="C40" s="31">
+        <v>46082</v>
+      </c>
+      <c r="D40" s="4">
+        <v>0</v>
+      </c>
+      <c r="E40" s="18">
+        <v>0</v>
+      </c>
+      <c r="F40" s="4">
+        <v>500</v>
+      </c>
+      <c r="G40" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="H40" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="I40" s="4">
+        <v>0</v>
+      </c>
+      <c r="J40" s="4"/>
+      <c r="K40" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="4"/>
+      <c r="B41" s="29">
+        <v>7</v>
+      </c>
+      <c r="C41" s="31">
+        <v>46081</v>
+      </c>
+      <c r="D41" s="4">
+        <v>0</v>
+      </c>
+      <c r="E41" s="18">
+        <v>0</v>
+      </c>
+      <c r="F41" s="4">
+        <v>500</v>
+      </c>
+      <c r="G41" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>77</v>
+      </c>
+      <c r="H41" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="I41" s="4">
+        <v>0</v>
+      </c>
+      <c r="J41" s="4">
+        <v>2</v>
+      </c>
+      <c r="K41" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" s="4"/>
+      <c r="B42" s="29">
+        <v>8</v>
+      </c>
+      <c r="C42" s="31">
+        <v>46080</v>
+      </c>
+      <c r="D42" s="4">
+        <v>0</v>
+      </c>
+      <c r="E42" s="18">
+        <v>1</v>
+      </c>
+      <c r="F42" s="4">
+        <v>500</v>
+      </c>
+      <c r="G42" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>81</v>
+      </c>
+      <c r="H42" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="I42" s="4">
+        <v>6</v>
+      </c>
+      <c r="J42" s="4"/>
+      <c r="K42" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" s="4"/>
+      <c r="B43" s="29">
+        <v>9</v>
+      </c>
+      <c r="C43" s="31">
+        <v>46079</v>
+      </c>
+      <c r="D43" s="4">
+        <v>10000</v>
+      </c>
+      <c r="E43" s="18">
+        <v>1</v>
+      </c>
+      <c r="F43" s="4">
+        <v>500</v>
+      </c>
+      <c r="G43" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>62</v>
+      </c>
+      <c r="H43" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>52</v>
+      </c>
+      <c r="I43" s="4">
+        <v>0</v>
+      </c>
+      <c r="J43" s="4">
+        <v>2</v>
+      </c>
+      <c r="K43" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" s="4"/>
+      <c r="B44" s="29">
+        <v>10</v>
+      </c>
+      <c r="C44" s="31">
+        <v>46078</v>
+      </c>
+      <c r="D44" s="4">
+        <v>0</v>
+      </c>
+      <c r="E44" s="18">
+        <v>0</v>
+      </c>
+      <c r="F44" s="4">
+        <v>500</v>
+      </c>
+      <c r="G44" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="H44" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="I44" s="4">
+        <v>0</v>
+      </c>
+      <c r="J44" s="4"/>
+      <c r="K44" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" s="4"/>
+      <c r="B45" s="29">
+        <v>11</v>
+      </c>
+      <c r="C45" s="31">
+        <v>46077</v>
+      </c>
+      <c r="D45" s="4">
+        <v>0</v>
+      </c>
+      <c r="E45" s="18">
+        <v>1</v>
+      </c>
+      <c r="F45" s="4">
+        <v>500</v>
+      </c>
+      <c r="G45" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>96</v>
+      </c>
+      <c r="H45" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="I45" s="4">
+        <v>0</v>
+      </c>
+      <c r="J45" s="4">
+        <v>2</v>
+      </c>
+      <c r="K45" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" s="4"/>
+      <c r="B46" s="29">
+        <v>12</v>
+      </c>
+      <c r="C46" s="31">
+        <v>46076</v>
+      </c>
+      <c r="D46" s="4">
+        <v>0</v>
+      </c>
+      <c r="E46" s="18">
+        <v>1</v>
+      </c>
+      <c r="F46" s="4">
+        <v>500</v>
+      </c>
+      <c r="G46" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>33</v>
+      </c>
+      <c r="H46" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>43</v>
+      </c>
+      <c r="I46" s="4">
+        <v>0</v>
+      </c>
+      <c r="J46" s="4"/>
+      <c r="K46" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" s="4"/>
+      <c r="B47" s="29">
+        <v>13</v>
+      </c>
+      <c r="C47" s="31">
+        <v>46075</v>
+      </c>
+      <c r="D47" s="4">
+        <v>0</v>
+      </c>
+      <c r="E47" s="18">
+        <v>1</v>
+      </c>
+      <c r="F47" s="4">
+        <v>500</v>
+      </c>
+      <c r="G47" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>29</v>
+      </c>
+      <c r="H47" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="I47" s="4">
+        <v>0</v>
+      </c>
+      <c r="J47" s="4">
+        <v>2</v>
+      </c>
+      <c r="K47" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" s="4"/>
+      <c r="B48" s="29">
+        <v>14</v>
+      </c>
+      <c r="C48" s="31">
+        <v>46074</v>
+      </c>
+      <c r="D48" s="4">
+        <v>0</v>
+      </c>
+      <c r="E48" s="18">
+        <v>1</v>
+      </c>
+      <c r="F48" s="4">
+        <v>500</v>
+      </c>
+      <c r="G48" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="H48" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>83</v>
+      </c>
+      <c r="I48" s="4">
+        <v>0</v>
+      </c>
+      <c r="J48" s="4"/>
+      <c r="K48" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" s="4"/>
+      <c r="B49" s="29">
+        <v>15</v>
+      </c>
+      <c r="C49" s="31">
+        <v>46073</v>
+      </c>
+      <c r="D49" s="4">
+        <v>0</v>
+      </c>
+      <c r="E49" s="18">
+        <v>0</v>
+      </c>
+      <c r="F49" s="4">
+        <v>500</v>
+      </c>
+      <c r="G49" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="H49" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="I49" s="4">
+        <v>6</v>
+      </c>
+      <c r="J49" s="4">
+        <v>2</v>
+      </c>
+      <c r="K49" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" s="4"/>
+      <c r="B50" s="29">
+        <v>16</v>
+      </c>
+      <c r="C50" s="31">
+        <v>46072</v>
+      </c>
+      <c r="D50" s="4">
+        <v>0</v>
+      </c>
+      <c r="E50" s="18">
+        <v>0</v>
+      </c>
+      <c r="F50" s="4">
+        <v>500</v>
+      </c>
+      <c r="G50" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H50" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="I50" s="4">
+        <v>0</v>
+      </c>
+      <c r="J50" s="4"/>
+      <c r="K50" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" s="4"/>
+      <c r="B51" s="29">
+        <v>17</v>
+      </c>
+      <c r="C51" s="31">
+        <v>46071</v>
+      </c>
+      <c r="D51" s="4">
+        <v>0</v>
+      </c>
+      <c r="E51" s="18">
+        <v>2</v>
+      </c>
+      <c r="F51" s="4">
+        <v>500</v>
+      </c>
+      <c r="G51" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>51</v>
+      </c>
+      <c r="H51" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>86</v>
+      </c>
+      <c r="I51" s="4">
+        <v>0</v>
+      </c>
+      <c r="J51" s="4">
+        <v>2</v>
+      </c>
+      <c r="K51" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B52" s="29">
+        <v>18</v>
+      </c>
+      <c r="C52" s="31">
+        <v>46070</v>
+      </c>
+      <c r="D52" s="4">
+        <v>0</v>
+      </c>
+      <c r="E52" s="18">
+        <v>1</v>
+      </c>
+      <c r="F52" s="4">
+        <v>500</v>
+      </c>
+      <c r="G52" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>74</v>
+      </c>
+      <c r="H52" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>63</v>
+      </c>
+      <c r="I52" s="4">
+        <v>0</v>
+      </c>
+      <c r="J52" s="4"/>
+      <c r="K52" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B53" s="29">
+        <v>19</v>
+      </c>
+      <c r="C53" s="31">
+        <v>46069</v>
+      </c>
+      <c r="D53" s="4">
+        <v>0</v>
+      </c>
+      <c r="E53" s="18">
+        <v>0</v>
+      </c>
+      <c r="F53" s="4">
+        <v>500</v>
+      </c>
+      <c r="G53" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>71</v>
+      </c>
+      <c r="H53" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>96</v>
+      </c>
+      <c r="I53" s="4">
+        <v>0</v>
+      </c>
+      <c r="J53" s="4">
+        <v>2</v>
+      </c>
+      <c r="K53" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B54" s="29">
+        <v>20</v>
+      </c>
+      <c r="C54" s="31">
+        <v>46068</v>
+      </c>
+      <c r="D54" s="4">
+        <v>0</v>
+      </c>
+      <c r="E54" s="18">
+        <v>1</v>
+      </c>
+      <c r="F54" s="4">
+        <v>500</v>
+      </c>
+      <c r="G54" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="H54" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>37</v>
+      </c>
+      <c r="I54" s="4">
+        <v>0</v>
+      </c>
+      <c r="J54" s="4"/>
+      <c r="K54" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B55" s="29">
+        <v>21</v>
+      </c>
+      <c r="C55" s="31">
+        <v>46067</v>
+      </c>
+      <c r="D55" s="4">
+        <v>0</v>
+      </c>
+      <c r="E55" s="18">
+        <v>1</v>
+      </c>
+      <c r="F55" s="4">
+        <v>500</v>
+      </c>
+      <c r="G55" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="H55" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>66</v>
+      </c>
+      <c r="I55" s="4">
+        <v>0</v>
+      </c>
+      <c r="J55" s="4">
+        <v>2</v>
+      </c>
+      <c r="K55" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B56" s="29">
+        <v>22</v>
+      </c>
+      <c r="C56" s="31">
+        <v>46066</v>
+      </c>
+      <c r="D56" s="4">
+        <v>0</v>
+      </c>
+      <c r="E56" s="18">
+        <v>1</v>
+      </c>
+      <c r="F56" s="4">
+        <v>500</v>
+      </c>
+      <c r="G56" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="H56" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>76</v>
+      </c>
+      <c r="I56" s="4">
+        <v>6</v>
+      </c>
+      <c r="J56" s="4"/>
+      <c r="K56" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B57" s="29">
+        <v>23</v>
+      </c>
+      <c r="C57" s="31">
+        <v>46065</v>
+      </c>
+      <c r="D57" s="4">
+        <v>0</v>
+      </c>
+      <c r="E57" s="18">
+        <v>3</v>
+      </c>
+      <c r="F57" s="4">
+        <v>500</v>
+      </c>
+      <c r="G57" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="H57" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="I57" s="4">
+        <v>0</v>
+      </c>
+      <c r="J57" s="4">
+        <v>2</v>
+      </c>
+      <c r="K57" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B58" s="29">
+        <v>24</v>
+      </c>
+      <c r="C58" s="31">
+        <v>46064</v>
+      </c>
+      <c r="D58" s="4">
+        <v>0</v>
+      </c>
+      <c r="E58" s="18">
+        <v>0</v>
+      </c>
+      <c r="F58" s="4">
+        <v>500</v>
+      </c>
+      <c r="G58" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>63</v>
+      </c>
+      <c r="H58" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="I58" s="4">
+        <v>0</v>
+      </c>
+      <c r="J58" s="4"/>
+      <c r="K58" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B59" s="29">
+        <v>25</v>
+      </c>
+      <c r="C59" s="31">
+        <v>46063</v>
+      </c>
+      <c r="D59" s="4">
+        <v>0</v>
+      </c>
+      <c r="E59" s="18">
+        <v>0</v>
+      </c>
+      <c r="F59" s="4">
+        <v>500</v>
+      </c>
+      <c r="G59" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H59" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>60</v>
+      </c>
+      <c r="I59" s="4">
+        <v>0</v>
+      </c>
+      <c r="J59" s="4">
+        <v>2</v>
+      </c>
+      <c r="K59" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B60" s="29">
+        <v>26</v>
+      </c>
+      <c r="C60" s="31">
+        <v>46062</v>
+      </c>
+      <c r="D60" s="4">
+        <v>0</v>
+      </c>
+      <c r="E60" s="18">
+        <v>1</v>
+      </c>
+      <c r="F60" s="4">
+        <v>500</v>
+      </c>
+      <c r="G60" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H60" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>82</v>
+      </c>
+      <c r="I60" s="4">
+        <v>0</v>
+      </c>
+      <c r="J60" s="4"/>
+      <c r="K60" s="18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B61" s="29">
+        <v>27</v>
+      </c>
+      <c r="C61" s="31">
+        <v>46061</v>
+      </c>
+      <c r="D61" s="4">
+        <v>0</v>
+      </c>
+      <c r="E61" s="18">
+        <v>0</v>
+      </c>
+      <c r="F61" s="4">
+        <v>500</v>
+      </c>
+      <c r="G61" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="H61" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>51</v>
+      </c>
+      <c r="I61" s="4">
+        <v>0</v>
+      </c>
+      <c r="J61" s="4">
+        <v>0</v>
+      </c>
+      <c r="K61" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B62" s="29">
+        <v>28</v>
+      </c>
+      <c r="C62" s="31">
+        <v>46060</v>
+      </c>
+      <c r="D62" s="4">
+        <v>0</v>
+      </c>
+      <c r="E62" s="18">
+        <v>0</v>
+      </c>
+      <c r="F62" s="4">
+        <v>500</v>
+      </c>
+      <c r="G62" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>87</v>
+      </c>
+      <c r="H62" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>80</v>
+      </c>
+      <c r="I62" s="4">
+        <v>0</v>
+      </c>
+      <c r="J62" s="4">
+        <v>0</v>
+      </c>
+      <c r="K62" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B63" s="29">
+        <v>29</v>
+      </c>
+      <c r="C63" s="31">
+        <v>46059</v>
+      </c>
+      <c r="D63" s="4">
+        <v>0</v>
+      </c>
+      <c r="E63" s="18">
+        <v>3</v>
+      </c>
+      <c r="F63" s="4">
+        <v>500</v>
+      </c>
+      <c r="G63" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="H63" s="4">
+        <f t="shared" ca="1" si="0"/>
+        <v>51</v>
+      </c>
+      <c r="I63" s="4">
+        <v>6</v>
+      </c>
+      <c r="J63" s="4">
+        <v>0</v>
+      </c>
+      <c r="K63" s="18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B64" s="30">
+        <v>30</v>
+      </c>
+      <c r="C64" s="32">
+        <v>46058</v>
+      </c>
+      <c r="D64" s="8">
+        <v>0</v>
+      </c>
+      <c r="E64" s="9">
+        <v>0</v>
+      </c>
+      <c r="F64" s="8">
+        <v>500</v>
+      </c>
+      <c r="G64" s="8">
+        <f ca="1">RANDBETWEEN(0,100)</f>
+        <v>43</v>
+      </c>
+      <c r="H64" s="8">
+        <f ca="1">RANDBETWEEN(0,100)</f>
+        <v>52</v>
+      </c>
+      <c r="I64" s="8">
+        <v>0</v>
+      </c>
+      <c r="J64" s="8">
+        <v>0</v>
+      </c>
+      <c r="K64" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C65" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D65" s="2">
+        <f>SUM(D35:D64)</f>
+        <v>10000</v>
+      </c>
+      <c r="E65" s="2">
+        <f t="shared" ref="E65:K65" si="1">SUM(E35:E64)</f>
+        <v>21</v>
+      </c>
+      <c r="F65" s="2">
+        <f t="shared" si="1"/>
+        <v>15000</v>
+      </c>
+      <c r="G65" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>1234</v>
+      </c>
+      <c r="H65" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>1526</v>
+      </c>
+      <c r="I65" s="2">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="J65" s="2">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+      <c r="K65" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="8">
     <mergeCell ref="B17:O17"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="B32:K32"/>
+    <mergeCell ref="B33:B34"/>
   </mergeCells>
+  <conditionalFormatting sqref="C35:C64">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>WEEKDAY(C35,2)&gt;5</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>